<commit_message>
Refactor Actions.txt to enhance SAP navigation documentation, including detailed screen flow and variable definitions. Update error handling to include HTML email notifications for login failures and improve row processing logic. Standardize Excel read operations to use ReadCellText for consistent data retrieval. Update frida-core.mdc with guidelines on indentation and reusable functions for better script organization.
</commit_message>
<xml_diff>
--- a/Inputs/COMPRA PERGAMINO ESPECIAL - 100126.xlsx
+++ b/Inputs/COMPRA PERGAMINO ESPECIAL - 100126.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodrigo.gracia\Documents\Projects\ECOM\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72AAB96A-56D9-4B30-B431-804FF9839BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B32A3ED-E12B-4962-91AE-687EBF36DC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-3210" yWindow="7570" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="121">
   <si>
     <t>ContractType</t>
   </si>
@@ -856,40 +856,61 @@
     <t>Chaparral</t>
   </si>
   <si>
+    <t>SUCCESS</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-02_14-48-32</t>
+  </si>
+  <si>
+    <t>Characteristics: SAP(E) [ZACM000]: Not found Future Closing Price in the transaction FDCS17</t>
+  </si>
+  <si>
+    <t>Price Details (Header):</t>
+  </si>
+  <si>
+    <t>Characteristics:</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-02_16-43-28</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-03_12-20-35</t>
+  </si>
+  <si>
+    <t>Processing</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Price Details (BID): SAP status could not be read (screen may have changed)</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-03_21-40-17</t>
+  </si>
+  <si>
+    <t>Texts: SAP(E) [ZACM000]: Fill required fields</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-03_21-43-42</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_00-10-26</t>
+  </si>
+  <si>
+    <t>Entry Screen: SAP status could not be read (screen may have changed)</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_00-37-20</t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Details</t>
   </si>
   <si>
-    <t>Success</t>
-  </si>
-  <si>
-    <t>SUCCESS</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-02_14-48-32</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>Characteristics: SAP(E) [ZACM000]: Not found Future Closing Price in the transaction FDCS17</t>
-  </si>
-  <si>
-    <t>Price Details (Header):</t>
-  </si>
-  <si>
-    <t>Characteristics:</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-02_16-43-28</t>
-  </si>
-  <si>
-    <t>Processing</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-03_12-20-35</t>
+    <t>SAPBot_2026-03-04_00-38-17</t>
   </si>
 </sst>
 </file>
@@ -1687,10 +1708,10 @@
         <v>45</v>
       </c>
       <c r="AV1" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="AW1" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:49" x14ac:dyDescent="0.25">
@@ -1805,7 +1826,10 @@
         <v>55</v>
       </c>
       <c r="AV2" t="s">
-        <v>104</v>
+        <v>110</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:49" x14ac:dyDescent="0.25">
@@ -1918,7 +1942,10 @@
         <v>55</v>
       </c>
       <c r="AV3" t="s">
-        <v>104</v>
+        <v>110</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:49" x14ac:dyDescent="0.25">
@@ -2031,7 +2058,10 @@
         <v>55</v>
       </c>
       <c r="AV4" t="s">
-        <v>104</v>
+        <v>110</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:49" x14ac:dyDescent="0.25">
@@ -2146,10 +2176,7 @@
         <v>55</v>
       </c>
       <c r="AV5" t="s">
-        <v>107</v>
-      </c>
-      <c r="AW5" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:49" x14ac:dyDescent="0.25">
@@ -2264,12 +2291,6 @@
       <c r="AU6" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="AV6" t="s">
-        <v>112</v>
-      </c>
-      <c r="AW6" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
@@ -2381,12 +2402,6 @@
       <c r="AU7" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="AV7" t="s">
-        <v>107</v>
-      </c>
-      <c r="AW7" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
@@ -2498,12 +2513,6 @@
       </c>
       <c r="AU8" s="24" t="s">
         <v>55</v>
-      </c>
-      <c r="AV8" t="s">
-        <v>107</v>
-      </c>
-      <c r="AW8" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:49" x14ac:dyDescent="0.25">
@@ -2534,7 +2543,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" style="1" customWidth="1"/>
@@ -2746,16 +2755,16 @@
         <v>2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C11" s="25">
         <v>46083.618217592593</v>
       </c>
       <c r="D11" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E11" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -2763,16 +2772,16 @@
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C12" s="25">
         <v>46083.619270833333</v>
       </c>
       <c r="D12" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -2780,16 +2789,16 @@
         <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C13" s="25">
         <v>46083.620370370372</v>
       </c>
       <c r="D13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -2803,10 +2812,10 @@
         <v>46083.620532407411</v>
       </c>
       <c r="D14" t="s">
+        <v>103</v>
+      </c>
+      <c r="E14" t="s">
         <v>106</v>
-      </c>
-      <c r="E14" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2820,10 +2829,10 @@
         <v>46083.621030092596</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E15" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -2837,10 +2846,10 @@
         <v>46083.621435185189</v>
       </c>
       <c r="D16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -2854,10 +2863,10 @@
         <v>46083.621747685182</v>
       </c>
       <c r="D17" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E17" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2871,10 +2880,10 @@
         <v>46083.697187500002</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E18" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -2888,7 +2897,7 @@
         <v>46083.697557870371</v>
       </c>
       <c r="D19" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E19" t="s">
         <v>96</v>
@@ -2905,6 +2914,9 @@
         <v>46083.697928240741</v>
       </c>
       <c r="D20" t="s">
+        <v>107</v>
+      </c>
+      <c r="E20" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2919,7 +2931,10 @@
         <v>46083.698217592595</v>
       </c>
       <c r="D21" t="s">
-        <v>111</v>
+        <v>107</v>
+      </c>
+      <c r="E21" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -2933,7 +2948,120 @@
         <v>46084.514606481483</v>
       </c>
       <c r="D22" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" t="s">
         <v>113</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>2</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="25">
+        <v>46084.903865740744</v>
+      </c>
+      <c r="D23" t="s">
+        <v>112</v>
+      </c>
+      <c r="E23" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>2</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="25">
+        <v>46084.906307870369</v>
+      </c>
+      <c r="D24" t="s">
+        <v>114</v>
+      </c>
+      <c r="E24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>2</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="25">
+        <v>46085.008275462962</v>
+      </c>
+      <c r="D25" t="s">
+        <v>115</v>
+      </c>
+      <c r="E25" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>3</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="25">
+        <v>46085.009108796294</v>
+      </c>
+      <c r="D26" t="s">
+        <v>115</v>
+      </c>
+      <c r="E26" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>4</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="25">
+        <v>46085.009942129633</v>
+      </c>
+      <c r="D27" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>1</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="25">
+        <v>46085.026226851849</v>
+      </c>
+      <c r="D28" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>2</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" s="25">
+        <v>46085.027592592596</v>
+      </c>
+      <c r="D29" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Actions.txt to modify SAP SelectComboBox paths for CO-Purchase rules, ensuring correct screen navigation and data handling. Adjusted multiple entries to reflect new identifiers for improved processing accuracy.
</commit_message>
<xml_diff>
--- a/Inputs/COMPRA PERGAMINO ESPECIAL - 100126.xlsx
+++ b/Inputs/COMPRA PERGAMINO ESPECIAL - 100126.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodrigo.gracia\Documents\Projects\ECOM\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B32A3ED-E12B-4962-91AE-687EBF36DC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F76016-451D-484B-A6C2-617A3B36E7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-3210" yWindow="7570" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="126">
   <si>
     <t>ContractType</t>
   </si>
@@ -877,40 +877,55 @@
     <t>SAPBot_2026-03-03_12-20-35</t>
   </si>
   <si>
-    <t>Processing</t>
+    <t>Price Details (BID): SAP status could not be read (screen may have changed)</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-03_21-40-17</t>
+  </si>
+  <si>
+    <t>Texts: SAP(E) [ZACM000]: Fill required fields</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-03_21-43-42</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_00-10-26</t>
+  </si>
+  <si>
+    <t>Entry Screen: SAP status could not be read (screen may have changed)</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_00-37-20</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_00-38-17</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_01-43-54</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_02-19-46</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-03-04_02-21-50</t>
   </si>
   <si>
     <t>Failed</t>
   </si>
   <si>
-    <t>Price Details (BID): SAP status could not be read (screen may have changed)</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-03_21-40-17</t>
-  </si>
-  <si>
-    <t>Texts: SAP(E) [ZACM000]: Fill required fields</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-03_21-43-42</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-04_00-10-26</t>
-  </si>
-  <si>
-    <t>Entry Screen: SAP status could not be read (screen may have changed)</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-04_00-37-20</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Details</t>
-  </si>
-  <si>
-    <t>SAPBot_2026-03-04_00-38-17</t>
+    <t>Price Details (Header): SAP(E) [ZACM000]: Fill required fields</t>
+  </si>
+  <si>
+    <t>Characteristics: SAP(E) [ZACM000]: Fill required fields</t>
   </si>
 </sst>
 </file>
@@ -1826,10 +1841,7 @@
         <v>55</v>
       </c>
       <c r="AV2" t="s">
-        <v>110</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:49" x14ac:dyDescent="0.25">
@@ -1942,10 +1954,7 @@
         <v>55</v>
       </c>
       <c r="AV3" t="s">
-        <v>110</v>
-      </c>
-      <c r="AW3" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:49" x14ac:dyDescent="0.25">
@@ -2058,10 +2067,7 @@
         <v>55</v>
       </c>
       <c r="AV4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AW4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:49" x14ac:dyDescent="0.25">
@@ -2176,7 +2182,10 @@
         <v>55</v>
       </c>
       <c r="AV5" t="s">
-        <v>109</v>
+        <v>123</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:49" x14ac:dyDescent="0.25">
@@ -2291,6 +2300,12 @@
       <c r="AU6" s="24" t="s">
         <v>55</v>
       </c>
+      <c r="AV6" t="s">
+        <v>123</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
@@ -2402,6 +2417,12 @@
       <c r="AU7" s="24" t="s">
         <v>55</v>
       </c>
+      <c r="AV7" t="s">
+        <v>123</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
@@ -2513,6 +2534,12 @@
       </c>
       <c r="AU8" s="24" t="s">
         <v>55</v>
+      </c>
+      <c r="AV8" t="s">
+        <v>123</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:49" x14ac:dyDescent="0.25">
@@ -2543,7 +2570,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" style="1" customWidth="1"/>
@@ -2917,7 +2944,7 @@
         <v>107</v>
       </c>
       <c r="E20" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -2934,7 +2961,7 @@
         <v>107</v>
       </c>
       <c r="E21" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -2951,7 +2978,7 @@
         <v>108</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -2965,10 +2992,10 @@
         <v>46084.903865740744</v>
       </c>
       <c r="D23" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -2982,10 +3009,10 @@
         <v>46084.906307870369</v>
       </c>
       <c r="D24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E24" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -2999,10 +3026,10 @@
         <v>46085.008275462962</v>
       </c>
       <c r="D25" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E25" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -3016,10 +3043,10 @@
         <v>46085.009108796294</v>
       </c>
       <c r="D26" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E26" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -3033,7 +3060,10 @@
         <v>46085.009942129633</v>
       </c>
       <c r="D27" t="s">
-        <v>115</v>
+        <v>113</v>
+      </c>
+      <c r="E27" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3047,7 +3077,10 @@
         <v>46085.026226851849</v>
       </c>
       <c r="D28" t="s">
-        <v>117</v>
+        <v>115</v>
+      </c>
+      <c r="E28" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -3061,7 +3094,128 @@
         <v>46085.027592592596</v>
       </c>
       <c r="D29" t="s">
-        <v>120</v>
+        <v>116</v>
+      </c>
+      <c r="E29" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>2</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C30" s="25">
+        <v>46085.073171296295</v>
+      </c>
+      <c r="D30" t="s">
+        <v>117</v>
+      </c>
+      <c r="E30" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>2</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="25">
+        <v>46085.098194444443</v>
+      </c>
+      <c r="D31" t="s">
+        <v>121</v>
+      </c>
+      <c r="E31" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>3</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="25">
+        <v>46085.099594907406</v>
+      </c>
+      <c r="D32" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>4</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="25">
+        <v>46085.100462962961</v>
+      </c>
+      <c r="D33" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>5</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" s="25">
+        <v>46085.100624999999</v>
+      </c>
+      <c r="D34" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>6</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="25">
+        <v>46085.101053240738</v>
+      </c>
+      <c r="D35" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>7</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36" s="25">
+        <v>46085.101469907408</v>
+      </c>
+      <c r="D36" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>8</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" s="25">
+        <v>46085.101840277777</v>
+      </c>
+      <c r="D37" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>